<commit_message>
Redesign homepage: cursive Tangled title with crochet collage decorations
</commit_message>
<xml_diff>
--- a/projects.xlsx
+++ b/projects.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,61 +492,6 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Date_Created</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Christmas Tree</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>advsb</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>80</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>dv</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="n">
-        <v>2</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2025-12-16 12:11</t>
         </is>
       </c>
     </row>

</xml_diff>